<commit_message>
Update Comparativo Resultados XGBoost Regresión.xlsx
Update Comparativo Resultados XG
</commit_message>
<xml_diff>
--- a/Semana 3/Comparativo Resultados XGBoost Regresión.xlsx
+++ b/Semana 3/Comparativo Resultados XGBoost Regresión.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/60a5996fa5bd5176/Documentos/GitHub/MIAD_ML_NLP_2025/Semana 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{0CA9CE09-FE83-48B8-A750-9AD43226E008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02644388-049C-499D-8787-982A45894C3A}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="8_{0CA9CE09-FE83-48B8-A750-9AD43226E008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30645F9E-D80C-4883-98B8-C35532C25E13}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C814346A-01D5-4129-9633-7AEEF1D6FDD5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Enfoque</t>
   </si>
@@ -57,14 +57,76 @@
   </si>
   <si>
     <t>XGBoost con transformación logarítmica</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>XGBoost con Optimización Bayesiana</t>
+  </si>
+  <si>
+    <t>Búsqueda avanzada de hiperparámetros manteniendo todas las variables</t>
+  </si>
+  <si>
+    <t>XGBoost con Características Importantes</t>
+  </si>
+  <si>
+    <t>XGBoost con Características Filtradas</t>
+  </si>
+  <si>
+    <t>Selección sistemática de características con umbral de importancia mayor al 1%</t>
+  </si>
+  <si>
+    <t>Transformación logarítmica de la variable objetivo</t>
+  </si>
+  <si>
+    <t>XGBoost Solo Numérico</t>
+  </si>
+  <si>
+    <t>Eliminación de todas las variables categóricas</t>
+  </si>
+  <si>
+    <t>Parámetros por defecto</t>
+  </si>
+  <si>
+    <t>Ponderación por frecuencia de popularidad</t>
+  </si>
+  <si>
+    <t>Entrenamiento con parada temprana</t>
+  </si>
+  <si>
+    <t>Nro</t>
+  </si>
+  <si>
+    <t>Selección manual de características basada en importancia (las de mayor importancia, con los parámetros</t>
+  </si>
+  <si>
+    <t>Eliminación de variables de alta importancia + recorte de valores objetivo (5-95) + RandomizedSearchCV</t>
+  </si>
+  <si>
+    <t>Eliminación de variables de menor importancia + recorte de valores objetivo (5-95) + RandomizedSearchCV</t>
+  </si>
+  <si>
+    <t>Modelo XGBoost Optimizado (&lt; importancia)</t>
+  </si>
+  <si>
+    <t>Modelo XGBoost Optimizado (&gt; importancia)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -119,13 +181,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -143,6 +225,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -462,68 +548,193 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1069B7CD-4AEE-42D6-83A3-70FDB05091A2}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="33.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.26953125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="38.26953125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="53.26953125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="10.90625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="2">
+        <v>15.72</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="2">
+        <v>18.61</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="8">
         <v>3</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2">
+        <v>19.760000000000002</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2">
+        <v>19.78</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="2">
         <v>20.81</v>
       </c>
-      <c r="C2" s="3">
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="2">
         <v>8.7799999999999994</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="2">
+        <v>21.32</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="2">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="8">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="2">
+        <v>21.61</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="8">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2">
+        <v>22.31</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="2">
+        <v>9.34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="8">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3">
+      <c r="C11" s="2">
         <v>23.05</v>
       </c>
-      <c r="C3" s="3">
+      <c r="D11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="2">
         <v>9.41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="3">
-        <v>22.31</v>
-      </c>
-      <c r="C4" s="3">
-        <v>9.34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3">
-        <v>21.32</v>
-      </c>
-      <c r="C5" s="3">
-        <v>8.1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>